<commit_message>
docs: five-line headers on all docs and runs/ to model_runs/ path rewrites (2026-09-19/21 sessions)
</commit_message>
<xml_diff>
--- a/reports/cnn/FMD_Line_SixClasses_ResNet50_20260917.xlsx
+++ b/reports/cnn/FMD_Line_SixClasses_ResNet50_20260917.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\02-SSA\fmd-analysis\reports\cnn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BB522DB-5CB0-4C8C-A5A3-9632EBD817B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F957E531-B8CD-4354-8D0E-6AC2A3B90EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,10 +22,21 @@
     <sheet name="L31" sheetId="6" r:id="rId7"/>
     <sheet name="Cells by support" sheetId="7" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -163,6 +174,198 @@
     <t>Reading: a class-line cell with four or fewer test pictures carries almost no information (median F1 zero), a cell with 25 or more never scores zero, and every difference between the five lines sits inside those bands rather than in the line.</t>
   </si>
   <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>Overall Accuracy (%)</t>
+  </si>
+  <si>
+    <t>Macro recall (%)</t>
+  </si>
+  <si>
+    <t>Test images</t>
+  </si>
+  <si>
+    <t>Recall (%)</t>
+  </si>
+  <si>
+    <t>Training time (s)</t>
+  </si>
+  <si>
+    <t>Inference Time per Image(ms)</t>
+  </si>
+  <si>
+    <t>BB</t>
+  </si>
+  <si>
+    <t>BC</t>
+  </si>
+  <si>
+    <t>BI</t>
+  </si>
+  <si>
+    <t>B123</t>
+  </si>
+  <si>
+    <t>BOE</t>
+  </si>
+  <si>
+    <t>BS</t>
+  </si>
+  <si>
+    <t>COC</t>
+  </si>
+  <si>
+    <t>DC</t>
+  </si>
+  <si>
+    <t>DS</t>
+  </si>
+  <si>
+    <t>EP</t>
+  </si>
+  <si>
+    <t>FB</t>
+  </si>
+  <si>
+    <t>FM</t>
+  </si>
+  <si>
+    <t>HF</t>
+  </si>
+  <si>
+    <t>HO</t>
+  </si>
+  <si>
+    <t>LOC</t>
+  </si>
+  <si>
+    <t>LDO</t>
+  </si>
+  <si>
+    <t>ML</t>
+  </si>
+  <si>
+    <t>MPP</t>
+  </si>
+  <si>
+    <t>MUL</t>
+  </si>
+  <si>
+    <t>PM</t>
+  </si>
+  <si>
+    <t>VO</t>
+  </si>
+  <si>
+    <t>WP</t>
+  </si>
+  <si>
+    <t>ResNet50</t>
+  </si>
+  <si>
+    <t>The All five row adds the five confusion matrices together rather than averaging five numbers. Its accuracy, 96.26 percent, is over every test picture the run scored, and each class recall there is over all the test pictures of that class on all five lines. Its macro recall is the mean over the 6 classes of that pooled matrix, 93.58 percent, so it is a different quantity from the plain mean of the five per-line macro recalls, 75.96 percent, which appears on the Summary sheet.</t>
+  </si>
+  <si>
+    <t>Every line carries the same 6 classes, so a class absent from a line has no cells to report and its column is amber throughout.</t>
+  </si>
+  <si>
+    <t>Overall Accuracy is that line's own test half, so each figure rests on a different number of pictures: 690, 174, 257, 218, 132. Pooled over all 1471, accuracy is 96.26 percent; the plain mean of the five is 95.27 percent.</t>
+  </si>
+  <si>
+    <t>Macro recall is the mean of that line's per-class recalls, so a class with one or two test pictures moves it a lot. Accuracy and macro recall answer different questions and should be read together.</t>
+  </si>
+  <si>
+    <t>Dataset: the Updated folders plus the 177 pictures only the older library holds, one label per picture, exact-count stratified 70:30 inside each class inside each line, seed 42.</t>
+  </si>
+  <si>
+    <t>Input: the raw 2448x2048 frame resized to 224x224, no crop. Batch 4, 50 epochs, seed 42. This is not the crop pipeline of the six-architecture table, so the two are not directly comparable.</t>
+  </si>
+  <si>
+    <t>Training time and inference per image are that line's own run as recorded, in seconds and milliseconds. Inference was timed during the evaluation pass with no separate warmup pass, so it includes the one-time graph and cuDNN cost and reads higher than the warm column in the six-architecture table. Compare the two columns only with that in mind.</t>
+  </si>
+  <si>
+    <t>Every recall figure here is the row's true-class recall from that line's confusion matrix, on its own test half only. A cell with four or fewer test pictures is not evidence.</t>
+  </si>
+  <si>
+    <t>Scope: this workbook is the six classes the lead highlighted, Missing Primary Package, Multiple Lenses, Foreign Matter, Lens Off Center, Missing Lens and HEMA Obstruction, trained on their own with ResNet50. The sixteen other columns are amber because those classes were not part of this experiment, not because they were thin.</t>
+  </si>
+  <si>
+    <t>Legend: the short codes used in the Recall block above</t>
+  </si>
+  <si>
+    <t>(continued)</t>
+  </si>
+  <si>
+    <t>Bubble</t>
+  </si>
+  <si>
+    <t>Foreign Matter</t>
+  </si>
+  <si>
+    <t>Bubble Cluster</t>
+  </si>
+  <si>
+    <t>HEMA Fragment</t>
+  </si>
+  <si>
+    <t>Bubble Irregular</t>
+  </si>
+  <si>
+    <t>HEMA Obstruction</t>
+  </si>
+  <si>
+    <t>Bubble On 123</t>
+  </si>
+  <si>
+    <t>Lens Off Center</t>
+  </si>
+  <si>
+    <t>Bubble On Edge</t>
+  </si>
+  <si>
+    <t>Low Dose Obstructing Region of Interest</t>
+  </si>
+  <si>
+    <t>Bubble Scatter</t>
+  </si>
+  <si>
+    <t>Missing Lens</t>
+  </si>
+  <si>
+    <t>Cavity Off Center</t>
+  </si>
+  <si>
+    <t>Missing Primary Package</t>
+  </si>
+  <si>
+    <t>Dirty Camera</t>
+  </si>
+  <si>
+    <t>Multiple Lenses</t>
+  </si>
+  <si>
+    <t>Dirty Strobe</t>
+  </si>
+  <si>
+    <t>Package Misalignment</t>
+  </si>
+  <si>
+    <t>Extraneous Polymer</t>
+  </si>
+  <si>
+    <t>View Obstructed</t>
+  </si>
+  <si>
+    <t>Fiber</t>
+  </si>
+  <si>
+    <t>Wet Package</t>
+  </si>
+  <si>
     <t>L24: ResNet50, 70:30, batch 4, 50 epochs</t>
   </si>
   <si>
@@ -190,24 +393,6 @@
     <t>Note</t>
   </si>
   <si>
-    <t>Foreign Matter</t>
-  </si>
-  <si>
-    <t>HEMA Obstruction</t>
-  </si>
-  <si>
-    <t>Lens Off Center</t>
-  </si>
-  <si>
-    <t>Missing Lens</t>
-  </si>
-  <si>
-    <t>Missing Primary Package</t>
-  </si>
-  <si>
-    <t>Multiple Lenses</t>
-  </si>
-  <si>
     <t>Total</t>
   </si>
   <si>
@@ -275,187 +460,13 @@
   </si>
   <si>
     <t>thin</t>
-  </si>
-  <si>
-    <t>#</t>
-  </si>
-  <si>
-    <t>Model</t>
-  </si>
-  <si>
-    <t>Overall Accuracy (%)</t>
-  </si>
-  <si>
-    <t>Macro recall (%)</t>
-  </si>
-  <si>
-    <t>Test images</t>
-  </si>
-  <si>
-    <t>Recall (%)</t>
-  </si>
-  <si>
-    <t>Training time (s)</t>
-  </si>
-  <si>
-    <t>Inference Time per Image(ms)</t>
-  </si>
-  <si>
-    <t>BB</t>
-  </si>
-  <si>
-    <t>BC</t>
-  </si>
-  <si>
-    <t>BI</t>
-  </si>
-  <si>
-    <t>B123</t>
-  </si>
-  <si>
-    <t>BOE</t>
-  </si>
-  <si>
-    <t>BS</t>
-  </si>
-  <si>
-    <t>COC</t>
-  </si>
-  <si>
-    <t>DC</t>
-  </si>
-  <si>
-    <t>DS</t>
-  </si>
-  <si>
-    <t>EP</t>
-  </si>
-  <si>
-    <t>FB</t>
-  </si>
-  <si>
-    <t>FM</t>
-  </si>
-  <si>
-    <t>HF</t>
-  </si>
-  <si>
-    <t>HO</t>
-  </si>
-  <si>
-    <t>LOC</t>
-  </si>
-  <si>
-    <t>LDO</t>
-  </si>
-  <si>
-    <t>ML</t>
-  </si>
-  <si>
-    <t>MPP</t>
-  </si>
-  <si>
-    <t>MUL</t>
-  </si>
-  <si>
-    <t>PM</t>
-  </si>
-  <si>
-    <t>VO</t>
-  </si>
-  <si>
-    <t>WP</t>
-  </si>
-  <si>
-    <t>ResNet50</t>
-  </si>
-  <si>
-    <t>The All five row adds the five confusion matrices together rather than averaging five numbers. Its accuracy, 96.26 percent, is over every test picture the run scored, and each class recall there is over all the test pictures of that class on all five lines. Its macro recall is the mean over the 6 classes of that pooled matrix, 93.58 percent, so it is a different quantity from the plain mean of the five per-line macro recalls, 75.96 percent, which appears on the Summary sheet.</t>
-  </si>
-  <si>
-    <t>Every line carries the same 6 classes, so a class absent from a line has no cells to report and its column is amber throughout.</t>
-  </si>
-  <si>
-    <t>Overall Accuracy is that line's own test half, so each figure rests on a different number of pictures: 690, 174, 257, 218, 132. Pooled over all 1471, accuracy is 96.26 percent; the plain mean of the five is 95.27 percent.</t>
-  </si>
-  <si>
-    <t>Macro recall is the mean of that line's per-class recalls, so a class with one or two test pictures moves it a lot. Accuracy and macro recall answer different questions and should be read together.</t>
-  </si>
-  <si>
-    <t>Dataset: the Updated folders plus the 177 pictures only the older library holds, one label per picture, exact-count stratified 70:30 inside each class inside each line, seed 42.</t>
-  </si>
-  <si>
-    <t>Input: the raw 2448x2048 frame resized to 224x224, no crop. Batch 4, 50 epochs, seed 42. This is not the crop pipeline of the six-architecture table, so the two are not directly comparable.</t>
-  </si>
-  <si>
-    <t>Training time and inference per image are that line's own run as recorded, in seconds and milliseconds. Inference was timed during the evaluation pass with no separate warmup pass, so it includes the one-time graph and cuDNN cost and reads higher than the warm column in the six-architecture table. Compare the two columns only with that in mind.</t>
-  </si>
-  <si>
-    <t>Every recall figure here is the row's true-class recall from that line's confusion matrix, on its own test half only. A cell with four or fewer test pictures is not evidence.</t>
-  </si>
-  <si>
-    <t>Scope: this workbook is the six classes the lead highlighted, Missing Primary Package, Multiple Lenses, Foreign Matter, Lens Off Center, Missing Lens and HEMA Obstruction, trained on their own with ResNet50. The sixteen other columns are amber because those classes were not part of this experiment, not because they were thin.</t>
-  </si>
-  <si>
-    <t>Legend: the short codes used in the Recall block above</t>
-  </si>
-  <si>
-    <t>(continued)</t>
-  </si>
-  <si>
-    <t>Bubble</t>
-  </si>
-  <si>
-    <t>Bubble Cluster</t>
-  </si>
-  <si>
-    <t>HEMA Fragment</t>
-  </si>
-  <si>
-    <t>Bubble Irregular</t>
-  </si>
-  <si>
-    <t>Bubble On 123</t>
-  </si>
-  <si>
-    <t>Bubble On Edge</t>
-  </si>
-  <si>
-    <t>Low Dose Obstructing Region of Interest</t>
-  </si>
-  <si>
-    <t>Bubble Scatter</t>
-  </si>
-  <si>
-    <t>Cavity Off Center</t>
-  </si>
-  <si>
-    <t>Dirty Camera</t>
-  </si>
-  <si>
-    <t>Dirty Strobe</t>
-  </si>
-  <si>
-    <t>Package Misalignment</t>
-  </si>
-  <si>
-    <t>Extraneous Polymer</t>
-  </si>
-  <si>
-    <t>View Obstructed</t>
-  </si>
-  <si>
-    <t>Fiber</t>
-  </si>
-  <si>
-    <t>Wet Package</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -483,11 +494,6 @@
       <i/>
       <sz val="9"/>
       <color rgb="FF555555"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -536,7 +542,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -548,14 +554,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1049,73 +1054,73 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="62" customWidth="1"/>
     <col min="2" max="12" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1">
       <c r="A4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1">
       <c r="A5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1">
       <c r="A6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1">
       <c r="A9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1">
       <c r="A10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1">
       <c r="A11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1">
       <c r="A12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1">
       <c r="A14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1">
       <c r="A15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12">
       <c r="A17" s="2" t="s">
         <v>12</v>
       </c>
@@ -1153,7 +1158,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12">
       <c r="A18" s="3" t="s">
         <v>24</v>
       </c>
@@ -1191,7 +1196,7 @@
         <v>13.8</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12">
       <c r="A19" s="3" t="s">
         <v>25</v>
       </c>
@@ -1229,7 +1234,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12">
       <c r="A20" s="3" t="s">
         <v>26</v>
       </c>
@@ -1267,7 +1272,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12">
       <c r="A21" s="3" t="s">
         <v>27</v>
       </c>
@@ -1305,7 +1310,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12">
       <c r="A22" s="3" t="s">
         <v>28</v>
       </c>
@@ -1343,7 +1348,7 @@
         <v>2.9</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12">
       <c r="A23" s="5" t="s">
         <v>29</v>
       </c>
@@ -1373,17 +1378,17 @@
         <v>30.6</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12">
       <c r="A24" s="8" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12">
       <c r="A26" s="9" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12">
       <c r="A27" s="2" t="s">
         <v>32</v>
       </c>
@@ -1406,7 +1411,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12">
       <c r="A28" s="3" t="s">
         <v>39</v>
       </c>
@@ -1429,7 +1434,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12">
       <c r="A29" s="3" t="s">
         <v>40</v>
       </c>
@@ -1452,7 +1457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12">
       <c r="A30" s="3" t="s">
         <v>41</v>
       </c>
@@ -1475,7 +1480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12">
       <c r="A32" s="8" t="s">
         <v>42</v>
       </c>
@@ -1488,7 +1493,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:AD30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -1500,133 +1505,133 @@
     <col min="29" max="30" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="B1" s="13" t="s">
+    <row r="1" spans="1:30">
+      <c r="A1" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="G1" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13"/>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13"/>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
-      <c r="T1" s="13"/>
-      <c r="U1" s="13"/>
-      <c r="V1" s="13"/>
-      <c r="W1" s="13"/>
-      <c r="X1" s="13"/>
-      <c r="Y1" s="13"/>
-      <c r="Z1" s="13"/>
-      <c r="AA1" s="13"/>
-      <c r="AB1" s="13"/>
-      <c r="AC1" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="AD1" s="13" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
+      <c r="C1" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
+      <c r="T1" s="12"/>
+      <c r="U1" s="12"/>
+      <c r="V1" s="12"/>
+      <c r="W1" s="12"/>
+      <c r="X1" s="12"/>
+      <c r="Y1" s="12"/>
+      <c r="Z1" s="12"/>
+      <c r="AA1" s="12"/>
+      <c r="AB1" s="12"/>
+      <c r="AC1" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="AD1" s="12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:30">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
       <c r="G2" s="2" t="s">
-        <v>89</v>
+        <v>51</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>90</v>
+        <v>52</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>91</v>
+        <v>53</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>93</v>
+        <v>55</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>95</v>
+        <v>57</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>96</v>
+        <v>58</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>98</v>
+        <v>60</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>99</v>
+        <v>61</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>100</v>
+        <v>62</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>101</v>
+        <v>63</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>103</v>
+        <v>65</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>104</v>
+        <v>66</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>105</v>
+        <v>67</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>106</v>
+        <v>68</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>107</v>
+        <v>69</v>
       </c>
       <c r="Z2" s="2" t="s">
-        <v>108</v>
+        <v>70</v>
       </c>
       <c r="AA2" s="2" t="s">
-        <v>109</v>
+        <v>71</v>
       </c>
       <c r="AB2" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="AC2" s="13"/>
-      <c r="AD2" s="13"/>
-    </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="AC2" s="12"/>
+      <c r="AD2" s="12"/>
+    </row>
+    <row r="3" spans="1:30">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -1634,7 +1639,7 @@
         <v>24</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>111</v>
+        <v>73</v>
       </c>
       <c r="D3" s="3">
         <v>97.83</v>
@@ -1645,28 +1650,28 @@
       <c r="F3" s="3">
         <v>690</v>
       </c>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
       <c r="R3" s="3">
         <v>96.51</v>
       </c>
-      <c r="S3" s="11"/>
+      <c r="S3" s="10"/>
       <c r="T3" s="3">
         <v>95.56</v>
       </c>
       <c r="U3" s="3">
         <v>86.44</v>
       </c>
-      <c r="V3" s="11"/>
+      <c r="V3" s="10"/>
       <c r="W3" s="3">
         <v>100</v>
       </c>
@@ -1676,9 +1681,9 @@
       <c r="Y3" s="3">
         <v>98.02</v>
       </c>
-      <c r="Z3" s="11"/>
-      <c r="AA3" s="11"/>
-      <c r="AB3" s="11"/>
+      <c r="Z3" s="10"/>
+      <c r="AA3" s="10"/>
+      <c r="AB3" s="10"/>
       <c r="AC3" s="3">
         <v>828.9</v>
       </c>
@@ -1686,7 +1691,7 @@
         <v>5.1420000000000003</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -1694,7 +1699,7 @@
         <v>25</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>111</v>
+        <v>73</v>
       </c>
       <c r="D4" s="3">
         <v>95.98</v>
@@ -1705,28 +1710,28 @@
       <c r="F4" s="3">
         <v>174</v>
       </c>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="11"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
       <c r="R4" s="3">
         <v>100</v>
       </c>
-      <c r="S4" s="11"/>
+      <c r="S4" s="10"/>
       <c r="T4" s="3">
         <v>80</v>
       </c>
       <c r="U4" s="3">
         <v>0</v>
       </c>
-      <c r="V4" s="11"/>
+      <c r="V4" s="10"/>
       <c r="W4" s="3">
         <v>50</v>
       </c>
@@ -1736,9 +1741,9 @@
       <c r="Y4" s="3">
         <v>96.39</v>
       </c>
-      <c r="Z4" s="11"/>
-      <c r="AA4" s="11"/>
-      <c r="AB4" s="11"/>
+      <c r="Z4" s="10"/>
+      <c r="AA4" s="10"/>
+      <c r="AB4" s="10"/>
       <c r="AC4" s="3">
         <v>224.93</v>
       </c>
@@ -1746,7 +1751,7 @@
         <v>15.147</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -1754,7 +1759,7 @@
         <v>26</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>111</v>
+        <v>73</v>
       </c>
       <c r="D5" s="3">
         <v>94.55</v>
@@ -1765,28 +1770,28 @@
       <c r="F5" s="3">
         <v>257</v>
       </c>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="10"/>
       <c r="R5" s="3">
         <v>93.88</v>
       </c>
-      <c r="S5" s="11"/>
+      <c r="S5" s="10"/>
       <c r="T5" s="3">
         <v>0</v>
       </c>
       <c r="U5" s="3">
         <v>50</v>
       </c>
-      <c r="V5" s="11"/>
+      <c r="V5" s="10"/>
       <c r="W5" s="3">
         <v>0</v>
       </c>
@@ -1796,9 +1801,9 @@
       <c r="Y5" s="3">
         <v>96.04</v>
       </c>
-      <c r="Z5" s="11"/>
-      <c r="AA5" s="11"/>
-      <c r="AB5" s="11"/>
+      <c r="Z5" s="10"/>
+      <c r="AA5" s="10"/>
+      <c r="AB5" s="10"/>
       <c r="AC5" s="3">
         <v>322.31</v>
       </c>
@@ -1806,7 +1811,7 @@
         <v>10.728999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -1814,7 +1819,7 @@
         <v>27</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>111</v>
+        <v>73</v>
       </c>
       <c r="D6" s="3">
         <v>96.33</v>
@@ -1825,28 +1830,28 @@
       <c r="F6" s="3">
         <v>218</v>
       </c>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="10"/>
+      <c r="Q6" s="10"/>
       <c r="R6" s="3">
         <v>96.36</v>
       </c>
-      <c r="S6" s="11"/>
+      <c r="S6" s="10"/>
       <c r="T6" s="3">
         <v>0</v>
       </c>
       <c r="U6" s="3">
         <v>87.5</v>
       </c>
-      <c r="V6" s="11"/>
+      <c r="V6" s="10"/>
       <c r="W6" s="3">
         <v>100</v>
       </c>
@@ -1856,9 +1861,9 @@
       <c r="Y6" s="3">
         <v>100</v>
       </c>
-      <c r="Z6" s="11"/>
-      <c r="AA6" s="11"/>
-      <c r="AB6" s="11"/>
+      <c r="Z6" s="10"/>
+      <c r="AA6" s="10"/>
+      <c r="AB6" s="10"/>
       <c r="AC6" s="3">
         <v>283.39999999999998</v>
       </c>
@@ -1866,7 +1871,7 @@
         <v>12.166</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -1874,7 +1879,7 @@
         <v>28</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>111</v>
+        <v>73</v>
       </c>
       <c r="D7" s="3">
         <v>91.67</v>
@@ -1885,28 +1890,28 @@
       <c r="F7" s="3">
         <v>132</v>
       </c>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+      <c r="P7" s="10"/>
+      <c r="Q7" s="10"/>
       <c r="R7" s="3">
         <v>100</v>
       </c>
-      <c r="S7" s="11"/>
+      <c r="S7" s="10"/>
       <c r="T7" s="3">
         <v>0</v>
       </c>
       <c r="U7" s="3">
         <v>83.33</v>
       </c>
-      <c r="V7" s="11"/>
+      <c r="V7" s="10"/>
       <c r="W7" s="3">
         <v>100</v>
       </c>
@@ -1916,9 +1921,9 @@
       <c r="Y7" s="3">
         <v>68.97</v>
       </c>
-      <c r="Z7" s="11"/>
-      <c r="AA7" s="11"/>
-      <c r="AB7" s="11"/>
+      <c r="Z7" s="10"/>
+      <c r="AA7" s="10"/>
+      <c r="AB7" s="10"/>
       <c r="AC7" s="3">
         <v>175.92</v>
       </c>
@@ -1926,300 +1931,300 @@
         <v>10.965</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30">
       <c r="A9" s="8" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30">
       <c r="A10" s="8" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30">
       <c r="A11" s="8" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30">
       <c r="A12" s="8" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:30">
       <c r="A13" s="8" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:30">
       <c r="A14" s="8" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" spans="1:30">
       <c r="A15" s="8" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30">
       <c r="A16" s="8" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
       <c r="A17" s="8" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
       <c r="A19" s="9" t="s">
-        <v>121</v>
+        <v>83</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H20" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="13"/>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H21" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="13"/>
+      <c r="L21" s="13"/>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B22" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="B20" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="10" t="s">
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H22" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="13"/>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="H23" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="I23" s="13"/>
+      <c r="J23" s="13"/>
+      <c r="K23" s="13"/>
+      <c r="L23" s="13"/>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="H24" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="I24" s="13"/>
+      <c r="J24" s="13"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="13"/>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="H25" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="I25" s="13"/>
+      <c r="J25" s="13"/>
+      <c r="K25" s="13"/>
+      <c r="L25" s="13"/>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
+      <c r="L26" s="13"/>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="H27" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="H20" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
-      <c r="L20" s="12"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="10" t="s">
+      <c r="I27" s="13"/>
+      <c r="J27" s="13"/>
+      <c r="K27" s="13"/>
+      <c r="L27" s="13"/>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="H21" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="I21" s="12"/>
-      <c r="J21" s="12"/>
-      <c r="K21" s="12"/>
-      <c r="L21" s="12"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="10" t="s">
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="H28" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="H22" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="I22" s="12"/>
-      <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
-      <c r="L22" s="12"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="10" t="s">
+      <c r="I28" s="13"/>
+      <c r="J28" s="13"/>
+      <c r="K28" s="13"/>
+      <c r="L28" s="13"/>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="H23" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="I23" s="12"/>
-      <c r="J23" s="12"/>
-      <c r="K23" s="12"/>
-      <c r="L23" s="12"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-      <c r="G24" s="10" t="s">
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H29" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="H24" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="I24" s="12"/>
-      <c r="J24" s="12"/>
-      <c r="K24" s="12"/>
-      <c r="L24" s="12"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="10" t="s">
+      <c r="I29" s="13"/>
+      <c r="J29" s="13"/>
+      <c r="K29" s="13"/>
+      <c r="L29" s="13"/>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="H25" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="I25" s="12"/>
-      <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
-      <c r="L25" s="12"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="10" t="s">
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="H30" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="H26" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="I26" s="12"/>
-      <c r="J26" s="12"/>
-      <c r="K26" s="12"/>
-      <c r="L26" s="12"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B27" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="H27" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="I27" s="12"/>
-      <c r="J27" s="12"/>
-      <c r="K27" s="12"/>
-      <c r="L27" s="12"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="H28" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="I28" s="12"/>
-      <c r="J28" s="12"/>
-      <c r="K28" s="12"/>
-      <c r="L28" s="12"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A29" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="H29" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="I29" s="12"/>
-      <c r="J29" s="12"/>
-      <c r="K29" s="12"/>
-      <c r="L29" s="12"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="H30" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="I30" s="12"/>
-      <c r="J30" s="12"/>
-      <c r="K30" s="12"/>
-      <c r="L30" s="12"/>
+      <c r="I30" s="13"/>
+      <c r="J30" s="13"/>
+      <c r="K30" s="13"/>
+      <c r="L30" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="31">
@@ -2262,50 +2267,50 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="18.75">
       <c r="A1" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>47</v>
+        <v>111</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>48</v>
+        <v>112</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="3" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B6" s="3">
         <v>86</v>
@@ -2321,9 +2326,9 @@
       </c>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8">
       <c r="A7" s="3" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B7" s="3">
         <v>45</v>
@@ -2339,9 +2344,9 @@
       </c>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8">
       <c r="A8" s="3" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="B8" s="3">
         <v>59</v>
@@ -2357,9 +2362,9 @@
       </c>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8">
       <c r="A9" s="3" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="B9" s="3">
         <v>55</v>
@@ -2375,9 +2380,9 @@
       </c>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8">
       <c r="A10" s="3" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="B10" s="3">
         <v>344</v>
@@ -2393,9 +2398,9 @@
       </c>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8">
       <c r="A11" s="3" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="B11" s="3">
         <v>101</v>
@@ -2411,48 +2416,48 @@
       </c>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="10">
+    <row r="12" spans="1:8">
+      <c r="A12" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="9">
         <v>690</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8">
       <c r="A14" s="9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" s="2" t="s">
-        <v>60</v>
+        <v>118</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" s="6" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B16" s="3">
         <v>83</v>
@@ -2476,9 +2481,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8">
       <c r="A17" s="6" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B17" s="3">
         <v>1</v>
@@ -2502,9 +2507,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8">
       <c r="A18" s="6" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="B18" s="3">
         <v>3</v>
@@ -2528,9 +2533,9 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8">
       <c r="A19" s="6" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="B19" s="3">
         <v>0</v>
@@ -2554,9 +2559,9 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8">
       <c r="A20" s="6" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="B20" s="3">
         <v>0</v>
@@ -2580,9 +2585,9 @@
         <v>344</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8">
       <c r="A21" s="6" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="B21" s="3">
         <v>0</v>
@@ -2606,9 +2611,9 @@
         <v>101</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8">
       <c r="A22" s="8" t="s">
-        <v>62</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -2620,50 +2625,50 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="18.75">
       <c r="A1" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>47</v>
+        <v>111</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>48</v>
+        <v>112</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="3" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B6" s="3">
         <v>25</v>
@@ -2679,9 +2684,9 @@
       </c>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8">
       <c r="A7" s="3" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B7" s="3">
         <v>5</v>
@@ -2697,9 +2702,9 @@
       </c>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8">
       <c r="A8" s="3" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="B8" s="3">
         <v>2</v>
@@ -2714,12 +2719,12 @@
         <v>0</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" s="3" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="B9" s="3">
         <v>2</v>
@@ -2734,12 +2739,12 @@
         <v>0.66669999999999996</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" s="3" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="B10" s="3">
         <v>57</v>
@@ -2755,9 +2760,9 @@
       </c>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8">
       <c r="A11" s="3" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="B11" s="3">
         <v>83</v>
@@ -2773,48 +2778,48 @@
       </c>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="10">
+    <row r="12" spans="1:8">
+      <c r="A12" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="9">
         <v>174</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8">
       <c r="A14" s="9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" s="2" t="s">
-        <v>60</v>
+        <v>118</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" s="6" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B16" s="3">
         <v>25</v>
@@ -2838,9 +2843,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8">
       <c r="A17" s="6" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B17" s="3">
         <v>0</v>
@@ -2864,9 +2869,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8">
       <c r="A18" s="6" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="B18" s="3">
         <v>1</v>
@@ -2890,9 +2895,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8">
       <c r="A19" s="6" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="B19" s="3">
         <v>0</v>
@@ -2916,9 +2921,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8">
       <c r="A20" s="6" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="B20" s="3">
         <v>0</v>
@@ -2942,9 +2947,9 @@
         <v>57</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8">
       <c r="A21" s="6" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="B21" s="3">
         <v>1</v>
@@ -2968,9 +2973,9 @@
         <v>83</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8">
       <c r="A22" s="8" t="s">
-        <v>66</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -2982,50 +2987,50 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="18.75">
       <c r="A1" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>47</v>
+        <v>111</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>48</v>
+        <v>112</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="3" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B6" s="3">
         <v>49</v>
@@ -3041,9 +3046,9 @@
       </c>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8">
       <c r="A7" s="3" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B7" s="3">
         <v>1</v>
@@ -3058,12 +3063,12 @@
         <v>0</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" s="3" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="B8" s="3">
         <v>2</v>
@@ -3078,12 +3083,12 @@
         <v>0.33329999999999999</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" s="3" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="B9" s="3">
         <v>1</v>
@@ -3098,12 +3103,12 @@
         <v>0</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" s="3" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="B10" s="3">
         <v>2</v>
@@ -3118,12 +3123,12 @@
         <v>0.8</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" s="3" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="B11" s="3">
         <v>202</v>
@@ -3139,48 +3144,48 @@
       </c>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="10">
+    <row r="12" spans="1:8">
+      <c r="A12" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="9">
         <v>257</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8">
       <c r="A14" s="9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" s="2" t="s">
-        <v>60</v>
+        <v>118</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" s="6" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B16" s="3">
         <v>46</v>
@@ -3204,9 +3209,9 @@
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8">
       <c r="A17" s="6" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B17" s="3">
         <v>0</v>
@@ -3230,9 +3235,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8">
       <c r="A18" s="6" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="B18" s="3">
         <v>1</v>
@@ -3256,9 +3261,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8">
       <c r="A19" s="6" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="B19" s="3">
         <v>0</v>
@@ -3282,9 +3287,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8">
       <c r="A20" s="6" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="B20" s="3">
         <v>0</v>
@@ -3308,9 +3313,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8">
       <c r="A21" s="6" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="B21" s="3">
         <v>7</v>
@@ -3334,9 +3339,9 @@
         <v>202</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8">
       <c r="A22" s="8" t="s">
-        <v>69</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -3348,50 +3353,50 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="18.75">
       <c r="A1" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>47</v>
+        <v>111</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>48</v>
+        <v>112</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="3" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B6" s="3">
         <v>165</v>
@@ -3407,9 +3412,9 @@
       </c>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8">
       <c r="A7" s="3" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B7" s="3">
         <v>1</v>
@@ -3424,12 +3429,12 @@
         <v>0</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" s="3" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="B8" s="3">
         <v>8</v>
@@ -3445,9 +3450,9 @@
       </c>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8">
       <c r="A9" s="3" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="B9" s="3">
         <v>24</v>
@@ -3463,9 +3468,9 @@
       </c>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8">
       <c r="A10" s="3" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="B10" s="3">
         <v>4</v>
@@ -3480,12 +3485,12 @@
         <v>1</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" s="3" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="B11" s="3">
         <v>16</v>
@@ -3501,48 +3506,48 @@
       </c>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="10">
+    <row r="12" spans="1:8">
+      <c r="A12" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="9">
         <v>218</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8">
       <c r="A14" s="9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" s="2" t="s">
-        <v>60</v>
+        <v>118</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" s="6" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B16" s="3">
         <v>159</v>
@@ -3566,9 +3571,9 @@
         <v>165</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8">
       <c r="A17" s="6" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B17" s="3">
         <v>1</v>
@@ -3592,9 +3597,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8">
       <c r="A18" s="6" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="B18" s="3">
         <v>1</v>
@@ -3618,9 +3623,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8">
       <c r="A19" s="6" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="B19" s="3">
         <v>0</v>
@@ -3644,9 +3649,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8">
       <c r="A20" s="6" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="B20" s="3">
         <v>0</v>
@@ -3670,9 +3675,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8">
       <c r="A21" s="6" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="B21" s="3">
         <v>0</v>
@@ -3696,9 +3701,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8">
       <c r="A22" s="8" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -3710,50 +3715,50 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="18.75">
       <c r="A1" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>47</v>
+        <v>111</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>48</v>
+        <v>112</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="3" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B6" s="3">
         <v>59</v>
@@ -3769,9 +3774,9 @@
       </c>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8">
       <c r="A7" s="3" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B7" s="3">
         <v>1</v>
@@ -3786,12 +3791,12 @@
         <v>0</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" s="3" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="B8" s="3">
         <v>6</v>
@@ -3807,9 +3812,9 @@
       </c>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8">
       <c r="A9" s="3" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="B9" s="3">
         <v>15</v>
@@ -3825,9 +3830,9 @@
       </c>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8">
       <c r="A10" s="3" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="B10" s="3">
         <v>22</v>
@@ -3843,9 +3848,9 @@
       </c>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8">
       <c r="A11" s="3" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="B11" s="3">
         <v>29</v>
@@ -3861,48 +3866,48 @@
       </c>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="10">
+    <row r="12" spans="1:8">
+      <c r="A12" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="9">
         <v>132</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8">
       <c r="A14" s="9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" s="2" t="s">
-        <v>60</v>
+        <v>118</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" s="6" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B16" s="3">
         <v>59</v>
@@ -3926,9 +3931,9 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8">
       <c r="A17" s="6" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B17" s="3">
         <v>0</v>
@@ -3952,9 +3957,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8">
       <c r="A18" s="6" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="B18" s="3">
         <v>1</v>
@@ -3978,9 +3983,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8">
       <c r="A19" s="6" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="B19" s="3">
         <v>0</v>
@@ -4004,9 +4009,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8">
       <c r="A20" s="6" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="B20" s="3">
         <v>0</v>
@@ -4030,9 +4035,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8">
       <c r="A21" s="6" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="B21" s="3">
         <v>4</v>
@@ -4056,9 +4061,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8">
       <c r="A22" s="8" t="s">
-        <v>75</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -4070,7 +4075,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -4078,40 +4083,40 @@
     <col min="4" max="7" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="18.75">
       <c r="A1" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" s="8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" s="2" t="s">
-        <v>47</v>
+        <v>111</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>46</v>
+        <v>110</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>78</v>
+        <v>136</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" s="3">
         <v>1</v>
       </c>
@@ -4119,7 +4124,7 @@
         <v>26</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="D5" s="3">
         <v>1</v>
@@ -4131,10 +4136,10 @@
         <v>0</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" s="3">
         <v>1</v>
       </c>
@@ -4142,7 +4147,7 @@
         <v>26</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
@@ -4154,10 +4159,10 @@
         <v>0</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" s="3">
         <v>1</v>
       </c>
@@ -4165,7 +4170,7 @@
         <v>27</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="D7" s="3">
         <v>1</v>
@@ -4177,10 +4182,10 @@
         <v>0</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" s="3">
         <v>1</v>
       </c>
@@ -4188,7 +4193,7 @@
         <v>28</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="D8" s="3">
         <v>1</v>
@@ -4200,10 +4205,10 @@
         <v>0</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" s="3">
         <v>2</v>
       </c>
@@ -4211,7 +4216,7 @@
         <v>25</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="D9" s="3">
         <v>2</v>
@@ -4223,10 +4228,10 @@
         <v>0</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" s="3">
         <v>2</v>
       </c>
@@ -4234,7 +4239,7 @@
         <v>25</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="D10" s="3">
         <v>2</v>
@@ -4246,10 +4251,10 @@
         <v>0.66669999999999996</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" s="3">
         <v>2</v>
       </c>
@@ -4257,7 +4262,7 @@
         <v>26</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="D11" s="3">
         <v>2</v>
@@ -4269,10 +4274,10 @@
         <v>0.33329999999999999</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
       <c r="A12" s="3">
         <v>2</v>
       </c>
@@ -4280,7 +4285,7 @@
         <v>26</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="D12" s="3">
         <v>2</v>
@@ -4292,10 +4297,10 @@
         <v>0.8</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
       <c r="A13" s="3">
         <v>4</v>
       </c>
@@ -4303,7 +4308,7 @@
         <v>27</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="D13" s="3">
         <v>4</v>
@@ -4315,10 +4320,10 @@
         <v>1</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
       <c r="A14" s="3">
         <v>5</v>
       </c>
@@ -4326,7 +4331,7 @@
         <v>25</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="D14" s="3">
         <v>5</v>
@@ -4339,7 +4344,7 @@
       </c>
       <c r="G14" s="3"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="A15" s="3">
         <v>6</v>
       </c>
@@ -4347,7 +4352,7 @@
         <v>28</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="D15" s="3">
         <v>6</v>
@@ -4360,7 +4365,7 @@
       </c>
       <c r="G15" s="3"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="A16" s="3">
         <v>8</v>
       </c>
@@ -4368,7 +4373,7 @@
         <v>27</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="D16" s="3">
         <v>8</v>
@@ -4381,7 +4386,7 @@
       </c>
       <c r="G16" s="3"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -4389,7 +4394,7 @@
         <v>28</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="D17" s="3">
         <v>15</v>
@@ -4402,7 +4407,7 @@
       </c>
       <c r="G17" s="3"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -4410,7 +4415,7 @@
         <v>27</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="D18" s="3">
         <v>16</v>
@@ -4423,7 +4428,7 @@
       </c>
       <c r="G18" s="3"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7">
       <c r="A19" s="3">
         <v>22</v>
       </c>
@@ -4431,7 +4436,7 @@
         <v>28</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="D19" s="3">
         <v>22</v>
@@ -4444,7 +4449,7 @@
       </c>
       <c r="G19" s="3"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7">
       <c r="A20" s="3">
         <v>24</v>
       </c>
@@ -4452,7 +4457,7 @@
         <v>27</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="D20" s="3">
         <v>24</v>
@@ -4465,7 +4470,7 @@
       </c>
       <c r="G20" s="3"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7">
       <c r="A21" s="3">
         <v>25</v>
       </c>
@@ -4473,7 +4478,7 @@
         <v>25</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="D21" s="3">
         <v>25</v>
@@ -4486,7 +4491,7 @@
       </c>
       <c r="G21" s="3"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7">
       <c r="A22" s="3">
         <v>29</v>
       </c>
@@ -4494,7 +4499,7 @@
         <v>28</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="D22" s="3">
         <v>29</v>
@@ -4507,7 +4512,7 @@
       </c>
       <c r="G22" s="3"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7">
       <c r="A23" s="3">
         <v>45</v>
       </c>
@@ -4515,7 +4520,7 @@
         <v>24</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="D23" s="3">
         <v>45</v>
@@ -4528,7 +4533,7 @@
       </c>
       <c r="G23" s="3"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7">
       <c r="A24" s="3">
         <v>49</v>
       </c>
@@ -4536,7 +4541,7 @@
         <v>26</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="D24" s="3">
         <v>49</v>
@@ -4549,7 +4554,7 @@
       </c>
       <c r="G24" s="3"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7">
       <c r="A25" s="3">
         <v>55</v>
       </c>
@@ -4557,7 +4562,7 @@
         <v>24</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="D25" s="3">
         <v>55</v>
@@ -4570,7 +4575,7 @@
       </c>
       <c r="G25" s="3"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7">
       <c r="A26" s="3">
         <v>57</v>
       </c>
@@ -4578,7 +4583,7 @@
         <v>25</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="D26" s="3">
         <v>57</v>
@@ -4591,7 +4596,7 @@
       </c>
       <c r="G26" s="3"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7">
       <c r="A27" s="3">
         <v>59</v>
       </c>
@@ -4599,7 +4604,7 @@
         <v>24</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="D27" s="3">
         <v>59</v>
@@ -4612,7 +4617,7 @@
       </c>
       <c r="G27" s="3"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7">
       <c r="A28" s="3">
         <v>59</v>
       </c>
@@ -4620,7 +4625,7 @@
         <v>28</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="D28" s="3">
         <v>59</v>
@@ -4633,7 +4638,7 @@
       </c>
       <c r="G28" s="3"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7">
       <c r="A29" s="3">
         <v>83</v>
       </c>
@@ -4641,7 +4646,7 @@
         <v>25</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="D29" s="3">
         <v>83</v>
@@ -4654,7 +4659,7 @@
       </c>
       <c r="G29" s="3"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7">
       <c r="A30" s="3">
         <v>86</v>
       </c>
@@ -4662,7 +4667,7 @@
         <v>24</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="D30" s="3">
         <v>86</v>
@@ -4675,7 +4680,7 @@
       </c>
       <c r="G30" s="3"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7">
       <c r="A31" s="3">
         <v>101</v>
       </c>
@@ -4683,7 +4688,7 @@
         <v>24</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="D31" s="3">
         <v>101</v>
@@ -4696,7 +4701,7 @@
       </c>
       <c r="G31" s="3"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7">
       <c r="A32" s="3">
         <v>165</v>
       </c>
@@ -4704,7 +4709,7 @@
         <v>27</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="D32" s="3">
         <v>165</v>
@@ -4717,7 +4722,7 @@
       </c>
       <c r="G32" s="3"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7">
       <c r="A33" s="3">
         <v>202</v>
       </c>
@@ -4725,7 +4730,7 @@
         <v>26</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="D33" s="3">
         <v>202</v>
@@ -4738,7 +4743,7 @@
       </c>
       <c r="G33" s="3"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7">
       <c r="A34" s="3">
         <v>344</v>
       </c>
@@ -4746,7 +4751,7 @@
         <v>24</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="D34" s="3">
         <v>344</v>

</xml_diff>